<commit_message>
fix: fix theme selection bug, add advanced settings, fix exam timing, update API
</commit_message>
<xml_diff>
--- a/edudex_quiz_server/tests/api.xlsx
+++ b/edudex_quiz_server/tests/api.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Edudex-Quiz\edudex_quiz_server\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19A95623-AD84-4705-A639-894837E5BDD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{095BE61F-AB6A-45EA-A15E-6A64E951CB8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Authen" sheetId="1" r:id="rId1"/>
+    <sheet name="SERVER - TEACHER" sheetId="1" r:id="rId1"/>
+    <sheet name="TEACHER - STUDENT" sheetId="4" r:id="rId2"/>
+    <sheet name="STUDENT - TEACHER" sheetId="5" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="28">
   <si>
     <t>#</t>
   </si>
@@ -140,12 +142,128 @@
   <si>
     <t>Chưa được phân công</t>
   </si>
+  <si>
+    <t>Đăng nhập</t>
+  </si>
+  <si>
+    <t>Chức năng</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>GET</t>
+  </si>
+  <si>
+    <t>{
+    "success": true,
+    "data": [
+        {
+            "seat_number": 1,
+            "exam_code": "0102001",
+            "student_code": "SV8315",
+            "full_name": "Hồ Lễ",
+            "subject_name": "Cơ sở dữ liệu"
+        },
+        {
+            "seat_number": 20,
+            "exam_code": "0102020",
+            "student_code": "SV1260",
+            "full_name": "Em. Doãn Ngân Hiếu",
+            "subject_name": "Cơ sở dữ liệu"
+        }
+    ]
+}</t>
+  </si>
+  <si>
+    <t>Lấy danh sách thí sinh</t>
+  </si>
+  <si>
+    <r>
+      <t>/api/exam-schedule/shifts/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="5"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </rPr>
+      <t>{{id ca thi}}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </rPr>
+      <t>/rooms/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="5"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </rPr>
+      <t>{{id phòng thi}}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </rPr>
+      <t>/students</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Accept:application/json
+Content-Type:application/json
+Authorization:copecute </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="5"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </rPr>
+      <t>{{token}}</t>
+    </r>
+  </si>
+  <si>
+    <t>{
+    "success": true,
+    "data": []
+}</t>
+  </si>
+  <si>
+    <t>Không có thí sinh hoặc không thành công</t>
+  </si>
+  <si>
+    <t>API GIAO TIẾP GIỮA SERVER - CLIENT TEACHER</t>
+  </si>
+  <si>
+    <t>API GIAO TIẾP GIỮA TEACHER CLIENT - STUDENT CLIENT</t>
+  </si>
+  <si>
+    <t>API GIAO TIẾP GIỮA STUDENT CLIENT - TEACHER CLIENT</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -154,12 +272,34 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <scheme val="major"/>
+    </font>
+    <font>
       <b/>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="5"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <scheme val="major"/>
     </font>
   </fonts>
   <fills count="2">
@@ -170,7 +310,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -178,28 +318,104 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -482,245 +698,557 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F24"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="4" width="29.59765625" customWidth="1"/>
-    <col min="5" max="5" width="34.59765625" customWidth="1"/>
-    <col min="6" max="6" width="25.09765625" customWidth="1"/>
+    <col min="1" max="2" width="8.796875" style="1"/>
+    <col min="3" max="5" width="29.59765625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="34.59765625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="25.09765625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="43.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3"/>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="1" spans="1:8" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="31.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
+      <c r="H2" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="10" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="69" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="4" t="s">
+      <c r="H3" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="78" x14ac:dyDescent="0.3">
+      <c r="A4" s="4"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="69" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="4" t="s">
+      <c r="H4" s="4"/>
+    </row>
+    <row r="5" spans="1:8" ht="78" x14ac:dyDescent="0.3">
+      <c r="A5" s="4"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="10" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
+      <c r="H5" s="4"/>
+    </row>
+    <row r="6" spans="1:8" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="4">
+        <v>2</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="4"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F8" s="9"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F9" s="9"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F10" s="9"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F11" s="9"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F12" s="9"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F13" s="9"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F14" s="9"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F15" s="9"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F16" s="9"/>
+    </row>
+    <row r="17" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F17" s="9"/>
+    </row>
+    <row r="18" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F18" s="9"/>
+    </row>
+    <row r="19" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F19" s="9"/>
+    </row>
+    <row r="20" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F20" s="9"/>
+    </row>
+    <row r="21" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F21" s="9"/>
+    </row>
+    <row r="22" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F22" s="9"/>
+    </row>
+    <row r="23" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F23" s="9"/>
+    </row>
+    <row r="24" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F24" s="9"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
+  <mergeCells count="13">
+    <mergeCell ref="H3:H5"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="C3:C5"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="D3:D5"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32EEDF3D-0DFF-445F-940A-8CAAC0004B0C}">
+  <dimension ref="A1:H22"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="8.796875" style="1"/>
+    <col min="3" max="5" width="29.59765625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="34.59765625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="25.09765625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.796875" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="78" x14ac:dyDescent="0.3">
+      <c r="A4" s="4"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" s="4"/>
+    </row>
+    <row r="5" spans="1:8" ht="78" x14ac:dyDescent="0.3">
+      <c r="A5" s="4"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="4"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F6" s="9"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F7" s="9"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F8" s="9"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F9" s="9"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F10" s="9"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F11" s="9"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F12" s="9"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F13" s="9"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F14" s="9"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F15" s="9"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F16" s="9"/>
+    </row>
+    <row r="17" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F17" s="9"/>
+    </row>
+    <row r="18" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F18" s="9"/>
+    </row>
+    <row r="19" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F19" s="9"/>
+    </row>
+    <row r="20" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F20" s="9"/>
+    </row>
+    <row r="21" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F21" s="9"/>
+    </row>
+    <row r="22" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F22" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="C3:C5"/>
+    <mergeCell ref="D3:D5"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="H3:H5"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08AECEAD-17EF-4A7A-84E5-56C63D9423E0}">
+  <dimension ref="A1:H22"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="8.796875" style="1"/>
+    <col min="3" max="5" width="29.59765625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="34.59765625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="25.09765625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.796875" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="78" x14ac:dyDescent="0.3">
+      <c r="A4" s="4"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" s="4"/>
+    </row>
+    <row r="5" spans="1:8" ht="78" x14ac:dyDescent="0.3">
+      <c r="A5" s="4"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="4"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F6" s="9"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F7" s="9"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F8" s="9"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F9" s="9"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F10" s="9"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F11" s="9"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F12" s="9"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F13" s="9"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F14" s="9"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F15" s="9"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F16" s="9"/>
+    </row>
+    <row r="17" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F17" s="9"/>
+    </row>
+    <row r="18" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F18" s="9"/>
+    </row>
+    <row r="19" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F19" s="9"/>
+    </row>
+    <row r="20" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F20" s="9"/>
+    </row>
+    <row r="21" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F21" s="9"/>
+    </row>
+    <row r="22" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F22" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="C3:C5"/>
+    <mergeCell ref="D3:D5"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="H3:H5"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>